<commit_message>
Remove date segment from IAB asset and parent codes
</commit_message>
<xml_diff>
--- a/outputs/new-assets-only/Fiix_IAB_New_Assets_A26.xlsx
+++ b/outputs/new-assets-only/Fiix_IAB_New_Assets_A26.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Import Sheet" sheetId="1" r:id="R23d1be5eab844d45"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Import Sheet" sheetId="1" r:id="R6428bf937dc9461f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -391,7 +391,7 @@
         <x:v>Rockwell Integrated Architecture Demo Wall</x:v>
       </x:c>
       <x:c r="B2" s="6" t="str">
-        <x:v>IAB-20261023-DEMO-ROOM</x:v>
+        <x:v>IAB-DEMO-ROOM</x:v>
       </x:c>
       <x:c r="C2" s="6" t="str">
         <x:v>Locations And Facilities</x:v>
@@ -432,11 +432,11 @@
         <x:v>PLC / Network Core Process Skid</x:v>
       </x:c>
       <x:c r="B3" s="6" t="str">
-        <x:v>IAB-20261023-SKID-01</x:v>
+        <x:v>IAB-SKID-01</x:v>
       </x:c>
       <x:c r="C3" s="6" t="str"/>
       <x:c r="D3" s="6" t="str">
-        <x:v>IAB-20261023-DEMO-ROOM</x:v>
+        <x:v>IAB-DEMO-ROOM</x:v>
       </x:c>
       <x:c r="E3" s="6" t="str">
         <x:v>Central PLC/network/power skid with CompactLogix-style controller, Ethernet switch/security appliance, 22 mm operator devices, protection devices, and field terminal blocks.</x:v>
@@ -471,11 +471,11 @@
         <x:v>VFD and Motion Drive Process Skid</x:v>
       </x:c>
       <x:c r="B4" s="6" t="str">
-        <x:v>IAB-20261023-SKID-02</x:v>
+        <x:v>IAB-SKID-02</x:v>
       </x:c>
       <x:c r="C4" s="6" t="str"/>
       <x:c r="D4" s="6" t="str">
-        <x:v>IAB-20261023-DEMO-ROOM</x:v>
+        <x:v>IAB-DEMO-ROOM</x:v>
       </x:c>
       <x:c r="E4" s="6" t="str">
         <x:v>Drive technology skid with PowerFlex 755TS VFD, Kinetix servo drive modules, branch protection, contactors, and distributed terminal blocks.</x:v>
@@ -510,11 +510,11 @@
         <x:v>GuardLogix HMI Safety Process Skid</x:v>
       </x:c>
       <x:c r="B5" s="6" t="str">
-        <x:v>IAB-20261023-SKID-03</x:v>
+        <x:v>IAB-SKID-03</x:v>
       </x:c>
       <x:c r="C5" s="6" t="str"/>
       <x:c r="D5" s="6" t="str">
-        <x:v>IAB-20261023-DEMO-ROOM</x:v>
+        <x:v>IAB-DEMO-ROOM</x:v>
       </x:c>
       <x:c r="E5" s="6" t="str">
         <x:v>HMI and safety automation skid with PanelView, Compact GuardLogix/CompactLogix class controller, safety I/O, ArmorBlock/field I/O, and operator controls.</x:v>
@@ -549,11 +549,11 @@
         <x:v>Servo Motion Safety Cell Skid</x:v>
       </x:c>
       <x:c r="B6" s="6" t="str">
-        <x:v>IAB-20261023-SKID-04</x:v>
+        <x:v>IAB-SKID-04</x:v>
       </x:c>
       <x:c r="C6" s="6" t="str"/>
       <x:c r="D6" s="6" t="str">
-        <x:v>IAB-20261023-DEMO-ROOM</x:v>
+        <x:v>IAB-DEMO-ROOM</x:v>
       </x:c>
       <x:c r="E6" s="6" t="str">
         <x:v>Motion cell skid with Kinetix class servo drive, servo motor/axis hardware, safety interlocks, safety switch/guard locking, POINT I/O, and terminal marshalling.</x:v>
@@ -588,11 +588,11 @@
         <x:v>Guarding / E-Stop Safety Demonstration Skid</x:v>
       </x:c>
       <x:c r="B7" s="6" t="str">
-        <x:v>IAB-20261023-SKID-05</x:v>
+        <x:v>IAB-SKID-05</x:v>
       </x:c>
       <x:c r="C7" s="6" t="str"/>
       <x:c r="D7" s="6" t="str">
-        <x:v>IAB-20261023-DEMO-ROOM</x:v>
+        <x:v>IAB-DEMO-ROOM</x:v>
       </x:c>
       <x:c r="E7" s="6" t="str">
         <x:v>Machine safety demonstration skid with zone E-stops, GuardShield light curtains, Guardmaster safety switches, ArmorBlock safety I/O, and safety/status lamps.</x:v>
@@ -627,11 +627,11 @@
         <x:v>Compact Machine Control and Drives Skid</x:v>
       </x:c>
       <x:c r="B8" s="6" t="str">
-        <x:v>IAB-20261023-SKID-06</x:v>
+        <x:v>IAB-SKID-06</x:v>
       </x:c>
       <x:c r="C8" s="6" t="str"/>
       <x:c r="D8" s="6" t="str">
-        <x:v>IAB-20261023-DEMO-ROOM</x:v>
+        <x:v>IAB-DEMO-ROOM</x:v>
       </x:c>
       <x:c r="E8" s="6" t="str">
         <x:v>Compact machine control skid with HMI, Stratix switch, PLC, distributed I/O, VFD/servo technology, power distribution, and linear actuator/motor load.</x:v>
@@ -666,11 +666,11 @@
         <x:v>SKID-01 - PLC / PAC</x:v>
       </x:c>
       <x:c r="B9" s="6" t="str">
-        <x:v>IAB-20261023-SKID-01-B010</x:v>
+        <x:v>IAB-SKID-01-B010</x:v>
       </x:c>
       <x:c r="C9" s="6" t="str"/>
       <x:c r="D9" s="6" t="str">
-        <x:v>IAB-20261023-SKID-01</x:v>
+        <x:v>IAB-SKID-01</x:v>
       </x:c>
       <x:c r="E9" s="6" t="str">
         <x:v>CompactLogix / CompactLogix-style controller with Ethernet and I/O rack visible near top</x:v>
@@ -705,11 +705,11 @@
         <x:v>SKID-01 - Industrial firewall / security appliance</x:v>
       </x:c>
       <x:c r="B10" s="6" t="str">
-        <x:v>IAB-20261023-SKID-01-B020</x:v>
+        <x:v>IAB-SKID-01-B020</x:v>
       </x:c>
       <x:c r="C10" s="6" t="str"/>
       <x:c r="D10" s="6" t="str">
-        <x:v>IAB-20261023-SKID-01</x:v>
+        <x:v>IAB-SKID-01</x:v>
       </x:c>
       <x:c r="E10" s="6" t="str">
         <x:v>Fortinet FortiGate industrial/security appliance on lower left</x:v>
@@ -744,11 +744,11 @@
         <x:v>SKID-01 - Industrial Ethernet switch</x:v>
       </x:c>
       <x:c r="B11" s="6" t="str">
-        <x:v>IAB-20261023-SKID-01-B030</x:v>
+        <x:v>IAB-SKID-01-B030</x:v>
       </x:c>
       <x:c r="C11" s="6" t="str"/>
       <x:c r="D11" s="6" t="str">
-        <x:v>IAB-20261023-SKID-01</x:v>
+        <x:v>IAB-SKID-01</x:v>
       </x:c>
       <x:c r="E11" s="6" t="str">
         <x:v>Small DIN-rail managed/unmanaged Ethernet switch adjacent to firewall</x:v>
@@ -783,11 +783,11 @@
         <x:v>SKID-01 - Circuit protection</x:v>
       </x:c>
       <x:c r="B12" s="6" t="str">
-        <x:v>IAB-20261023-SKID-01-B040</x:v>
+        <x:v>IAB-SKID-01-B040</x:v>
       </x:c>
       <x:c r="C12" s="6" t="str"/>
       <x:c r="D12" s="6" t="str">
-        <x:v>IAB-20261023-SKID-01</x:v>
+        <x:v>IAB-SKID-01</x:v>
       </x:c>
       <x:c r="E12" s="6" t="str">
         <x:v>Molded case breaker and DIN rail branch protection</x:v>
@@ -822,11 +822,11 @@
         <x:v>SKID-01 - 22 mm pushbuttons / pilot devices</x:v>
       </x:c>
       <x:c r="B13" s="6" t="str">
-        <x:v>IAB-20261023-SKID-01-B050</x:v>
+        <x:v>IAB-SKID-01-B050</x:v>
       </x:c>
       <x:c r="C13" s="6" t="str"/>
       <x:c r="D13" s="6" t="str">
-        <x:v>IAB-20261023-SKID-01</x:v>
+        <x:v>IAB-SKID-01</x:v>
       </x:c>
       <x:c r="E13" s="6" t="str">
         <x:v>Multi-color operator pushbuttons, illuminated indicators, mushroom E-stop</x:v>
@@ -861,11 +861,11 @@
         <x:v>SKID-01 - Terminal blocks / marshalling</x:v>
       </x:c>
       <x:c r="B14" s="6" t="str">
-        <x:v>IAB-20261023-SKID-01-B060</x:v>
+        <x:v>IAB-SKID-01-B060</x:v>
       </x:c>
       <x:c r="C14" s="6" t="str"/>
       <x:c r="D14" s="6" t="str">
-        <x:v>IAB-20261023-SKID-01</x:v>
+        <x:v>IAB-SKID-01</x:v>
       </x:c>
       <x:c r="E14" s="6" t="str">
         <x:v>DIN rail terminal block banks with patch field labeling</x:v>
@@ -900,11 +900,11 @@
         <x:v>SKID-02 - VFD</x:v>
       </x:c>
       <x:c r="B15" s="6" t="str">
-        <x:v>IAB-20261023-SKID-02-B010</x:v>
+        <x:v>IAB-SKID-02-B010</x:v>
       </x:c>
       <x:c r="C15" s="6" t="str"/>
       <x:c r="D15" s="6" t="str">
-        <x:v>IAB-20261023-SKID-02</x:v>
+        <x:v>IAB-SKID-02</x:v>
       </x:c>
       <x:c r="E15" s="6" t="str">
         <x:v>PowerFlex 755TS visible with HIM keypad</x:v>
@@ -939,11 +939,11 @@
         <x:v>SKID-02 - Servo drive</x:v>
       </x:c>
       <x:c r="B16" s="6" t="str">
-        <x:v>IAB-20261023-SKID-02-B020</x:v>
+        <x:v>IAB-SKID-02-B020</x:v>
       </x:c>
       <x:c r="C16" s="6" t="str"/>
       <x:c r="D16" s="6" t="str">
-        <x:v>IAB-20261023-SKID-02</x:v>
+        <x:v>IAB-SKID-02</x:v>
       </x:c>
       <x:c r="E16" s="6" t="str">
         <x:v>Two Kinetix servo drive modules visible at upper left</x:v>
@@ -978,11 +978,11 @@
         <x:v>SKID-02 - EtherNet/IP option cabling</x:v>
       </x:c>
       <x:c r="B17" s="6" t="str">
-        <x:v>IAB-20261023-SKID-02-B030</x:v>
+        <x:v>IAB-SKID-02-B030</x:v>
       </x:c>
       <x:c r="C17" s="6" t="str"/>
       <x:c r="D17" s="6" t="str">
-        <x:v>IAB-20261023-SKID-02</x:v>
+        <x:v>IAB-SKID-02</x:v>
       </x:c>
       <x:c r="E17" s="6" t="str">
         <x:v>EtherNet/IP cables into PowerFlex and Kinetix devices</x:v>
@@ -1017,11 +1017,11 @@
         <x:v>SKID-02 - Disconnect / breaker</x:v>
       </x:c>
       <x:c r="B18" s="6" t="str">
-        <x:v>IAB-20261023-SKID-02-B040</x:v>
+        <x:v>IAB-SKID-02-B040</x:v>
       </x:c>
       <x:c r="C18" s="6" t="str"/>
       <x:c r="D18" s="6" t="str">
-        <x:v>IAB-20261023-SKID-02</x:v>
+        <x:v>IAB-SKID-02</x:v>
       </x:c>
       <x:c r="E18" s="6" t="str">
         <x:v>DIN rail breaker and larger disconnect/protection device</x:v>
@@ -1056,11 +1056,11 @@
         <x:v>SKID-02 - Contactor / overload</x:v>
       </x:c>
       <x:c r="B19" s="6" t="str">
-        <x:v>IAB-20261023-SKID-02-B050</x:v>
+        <x:v>IAB-SKID-02-B050</x:v>
       </x:c>
       <x:c r="C19" s="6" t="str"/>
       <x:c r="D19" s="6" t="str">
-        <x:v>IAB-20261023-SKID-02</x:v>
+        <x:v>IAB-SKID-02</x:v>
       </x:c>
       <x:c r="E19" s="6" t="str">
         <x:v>Contactor/overload assemblies at lower left</x:v>
@@ -1095,11 +1095,11 @@
         <x:v>SKID-02 - Terminal blocks / distribution</x:v>
       </x:c>
       <x:c r="B20" s="6" t="str">
-        <x:v>IAB-20261023-SKID-02-B060</x:v>
+        <x:v>IAB-SKID-02-B060</x:v>
       </x:c>
       <x:c r="C20" s="6" t="str"/>
       <x:c r="D20" s="6" t="str">
-        <x:v>IAB-20261023-SKID-02</x:v>
+        <x:v>IAB-SKID-02</x:v>
       </x:c>
       <x:c r="E20" s="6" t="str">
         <x:v>Field terminal blocks at right and adjacent panel edges</x:v>
@@ -1134,11 +1134,11 @@
         <x:v>SKID-03 - PanelView operator terminal</x:v>
       </x:c>
       <x:c r="B21" s="6" t="str">
-        <x:v>IAB-20261023-SKID-03-B010</x:v>
+        <x:v>IAB-SKID-03-B010</x:v>
       </x:c>
       <x:c r="C21" s="6" t="str"/>
       <x:c r="D21" s="6" t="str">
-        <x:v>IAB-20261023-SKID-03</x:v>
+        <x:v>IAB-SKID-03</x:v>
       </x:c>
       <x:c r="E21" s="6" t="str">
         <x:v>Allen-Bradley PanelView-style HMI displaying station test screen</x:v>
@@ -1173,11 +1173,11 @@
         <x:v>SKID-03 - Safety PLC</x:v>
       </x:c>
       <x:c r="B22" s="6" t="str">
-        <x:v>IAB-20261023-SKID-03-B020</x:v>
+        <x:v>IAB-SKID-03-B020</x:v>
       </x:c>
       <x:c r="C22" s="6" t="str"/>
       <x:c r="D22" s="6" t="str">
-        <x:v>IAB-20261023-SKID-03</x:v>
+        <x:v>IAB-SKID-03</x:v>
       </x:c>
       <x:c r="E22" s="6" t="str">
         <x:v>Compact GuardLogix 5380 class controller with safety cards visible</x:v>
@@ -1212,11 +1212,11 @@
         <x:v>SKID-03 - Safety and standard I/O</x:v>
       </x:c>
       <x:c r="B23" s="6" t="str">
-        <x:v>IAB-20261023-SKID-03-B030</x:v>
+        <x:v>IAB-SKID-03-B030</x:v>
       </x:c>
       <x:c r="C23" s="6" t="str"/>
       <x:c r="D23" s="6" t="str">
-        <x:v>IAB-20261023-SKID-03</x:v>
+        <x:v>IAB-SKID-03</x:v>
       </x:c>
       <x:c r="E23" s="6" t="str">
         <x:v>Local 5069 I/O modules and field I/O blocks</x:v>
@@ -1251,11 +1251,11 @@
         <x:v>SKID-03 - Industrial computer / gateway</x:v>
       </x:c>
       <x:c r="B24" s="6" t="str">
-        <x:v>IAB-20261023-SKID-03-B040</x:v>
+        <x:v>IAB-SKID-03-B040</x:v>
       </x:c>
       <x:c r="C24" s="6" t="str"/>
       <x:c r="D24" s="6" t="str">
-        <x:v>IAB-20261023-SKID-03</x:v>
+        <x:v>IAB-SKID-03</x:v>
       </x:c>
       <x:c r="E24" s="6" t="str">
         <x:v>Small Allen-Bradley industrial computer or gateway beneath HMI</x:v>
@@ -1290,11 +1290,11 @@
         <x:v>SKID-03 - Managed Ethernet switch</x:v>
       </x:c>
       <x:c r="B25" s="6" t="str">
-        <x:v>IAB-20261023-SKID-03-B050</x:v>
+        <x:v>IAB-SKID-03-B050</x:v>
       </x:c>
       <x:c r="C25" s="6" t="str"/>
       <x:c r="D25" s="6" t="str">
-        <x:v>IAB-20261023-SKID-03</x:v>
+        <x:v>IAB-SKID-03</x:v>
       </x:c>
       <x:c r="E25" s="6" t="str">
         <x:v>Blue managed switch / network appliance at lower left</x:v>
@@ -1329,11 +1329,11 @@
         <x:v>SKID-03 - Selector switches / pushbuttons</x:v>
       </x:c>
       <x:c r="B26" s="6" t="str">
-        <x:v>IAB-20261023-SKID-03-B060</x:v>
+        <x:v>IAB-SKID-03-B060</x:v>
       </x:c>
       <x:c r="C26" s="6" t="str"/>
       <x:c r="D26" s="6" t="str">
-        <x:v>IAB-20261023-SKID-03</x:v>
+        <x:v>IAB-SKID-03</x:v>
       </x:c>
       <x:c r="E26" s="6" t="str">
         <x:v>Three-position selector switches and pushbuttons on black operator plate</x:v>
@@ -1368,11 +1368,11 @@
         <x:v>SKID-03 - Safety I/O block / M12 connectivity</x:v>
       </x:c>
       <x:c r="B27" s="6" t="str">
-        <x:v>IAB-20261023-SKID-03-B070</x:v>
+        <x:v>IAB-SKID-03-B070</x:v>
       </x:c>
       <x:c r="C27" s="6" t="str"/>
       <x:c r="D27" s="6" t="str">
-        <x:v>IAB-20261023-SKID-03</x:v>
+        <x:v>IAB-SKID-03</x:v>
       </x:c>
       <x:c r="E27" s="6" t="str">
         <x:v>M12 field I/O block with yellow safety leads</x:v>
@@ -1407,11 +1407,11 @@
         <x:v>SKID-04 - Servo drive</x:v>
       </x:c>
       <x:c r="B28" s="6" t="str">
-        <x:v>IAB-20261023-SKID-04-B010</x:v>
+        <x:v>IAB-SKID-04-B010</x:v>
       </x:c>
       <x:c r="C28" s="6" t="str"/>
       <x:c r="D28" s="6" t="str">
-        <x:v>IAB-20261023-SKID-04</x:v>
+        <x:v>IAB-SKID-04</x:v>
       </x:c>
       <x:c r="E28" s="6" t="str">
         <x:v>Kinetix drive module(s) and motor cabling feeding axis fixture</x:v>
@@ -1446,11 +1446,11 @@
         <x:v>SKID-04 - Servo motor / axis assembly</x:v>
       </x:c>
       <x:c r="B29" s="6" t="str">
-        <x:v>IAB-20261023-SKID-04-B020</x:v>
+        <x:v>IAB-SKID-04-B020</x:v>
       </x:c>
       <x:c r="C29" s="6" t="str"/>
       <x:c r="D29" s="6" t="str">
-        <x:v>IAB-20261023-SKID-04</x:v>
+        <x:v>IAB-SKID-04</x:v>
       </x:c>
       <x:c r="E29" s="6" t="str">
         <x:v>Servo motor and guarded linear/rotary test fixture</x:v>
@@ -1485,11 +1485,11 @@
         <x:v>SKID-04 - Distributed controller / I/O</x:v>
       </x:c>
       <x:c r="B30" s="6" t="str">
-        <x:v>IAB-20261023-SKID-04-B030</x:v>
+        <x:v>IAB-SKID-04-B030</x:v>
       </x:c>
       <x:c r="C30" s="6" t="str"/>
       <x:c r="D30" s="6" t="str">
-        <x:v>IAB-20261023-SKID-04</x:v>
+        <x:v>IAB-SKID-04</x:v>
       </x:c>
       <x:c r="E30" s="6" t="str">
         <x:v>POINT I/O rack and controller/safety modules visible at upper right</x:v>
@@ -1524,11 +1524,11 @@
         <x:v>SKID-04 - Guard locking / safety switch</x:v>
       </x:c>
       <x:c r="B31" s="6" t="str">
-        <x:v>IAB-20261023-SKID-04-B040</x:v>
+        <x:v>IAB-SKID-04-B040</x:v>
       </x:c>
       <x:c r="C31" s="6" t="str"/>
       <x:c r="D31" s="6" t="str">
-        <x:v>IAB-20261023-SKID-04</x:v>
+        <x:v>IAB-SKID-04</x:v>
       </x:c>
       <x:c r="E31" s="6" t="str">
         <x:v>Red Guardmaster-style safety locking/safety switch on guard door</x:v>
@@ -1563,11 +1563,11 @@
         <x:v>SKID-04 - Safety interlock sensor</x:v>
       </x:c>
       <x:c r="B32" s="6" t="str">
-        <x:v>IAB-20261023-SKID-04-B050</x:v>
+        <x:v>IAB-SKID-04-B050</x:v>
       </x:c>
       <x:c r="C32" s="6" t="str"/>
       <x:c r="D32" s="6" t="str">
-        <x:v>IAB-20261023-SKID-04</x:v>
+        <x:v>IAB-SKID-04</x:v>
       </x:c>
       <x:c r="E32" s="6" t="str">
         <x:v>Red safety sensor/actuator mounted to sliding guard</x:v>
@@ -1602,11 +1602,11 @@
         <x:v>SKID-04 - Pushbutton / E-stop station</x:v>
       </x:c>
       <x:c r="B33" s="6" t="str">
-        <x:v>IAB-20261023-SKID-04-B060</x:v>
+        <x:v>IAB-SKID-04-B060</x:v>
       </x:c>
       <x:c r="C33" s="6" t="str"/>
       <x:c r="D33" s="6" t="str">
-        <x:v>IAB-20261023-SKID-04</x:v>
+        <x:v>IAB-SKID-04</x:v>
       </x:c>
       <x:c r="E33" s="6" t="str">
         <x:v>Pushbutton station with red/blue/black/E-stop buttons</x:v>
@@ -1641,11 +1641,11 @@
         <x:v>SKID-04 - Terminal blocks / safety marshalling</x:v>
       </x:c>
       <x:c r="B34" s="6" t="str">
-        <x:v>IAB-20261023-SKID-04-B070</x:v>
+        <x:v>IAB-SKID-04-B070</x:v>
       </x:c>
       <x:c r="C34" s="6" t="str"/>
       <x:c r="D34" s="6" t="str">
-        <x:v>IAB-20261023-SKID-04</x:v>
+        <x:v>IAB-SKID-04</x:v>
       </x:c>
       <x:c r="E34" s="6" t="str">
         <x:v>Field terminal blocks on right with safety/standard wiring</x:v>
@@ -1680,11 +1680,11 @@
         <x:v>SKID-05 - Safety light curtains</x:v>
       </x:c>
       <x:c r="B35" s="6" t="str">
-        <x:v>IAB-20261023-SKID-05-B010</x:v>
+        <x:v>IAB-SKID-05-B010</x:v>
       </x:c>
       <x:c r="C35" s="6" t="str"/>
       <x:c r="D35" s="6" t="str">
-        <x:v>IAB-20261023-SKID-05</x:v>
+        <x:v>IAB-SKID-05</x:v>
       </x:c>
       <x:c r="E35" s="6" t="str">
         <x:v>Two Allen-Bradley GuardShield light curtain columns</x:v>
@@ -1719,11 +1719,11 @@
         <x:v>SKID-05 - Guardmaster safety interlocks</x:v>
       </x:c>
       <x:c r="B36" s="6" t="str">
-        <x:v>IAB-20261023-SKID-05-B020</x:v>
+        <x:v>IAB-SKID-05-B020</x:v>
       </x:c>
       <x:c r="C36" s="6" t="str"/>
       <x:c r="D36" s="6" t="str">
-        <x:v>IAB-20261023-SKID-05</x:v>
+        <x:v>IAB-SKID-05</x:v>
       </x:c>
       <x:c r="E36" s="6" t="str">
         <x:v>Multiple red Guardmaster safety switch/sensor devices</x:v>
@@ -1758,11 +1758,11 @@
         <x:v>SKID-05 - Zone E-stops</x:v>
       </x:c>
       <x:c r="B37" s="6" t="str">
-        <x:v>IAB-20261023-SKID-05-B030</x:v>
+        <x:v>IAB-SKID-05-B030</x:v>
       </x:c>
       <x:c r="C37" s="6" t="str"/>
       <x:c r="D37" s="6" t="str">
-        <x:v>IAB-20261023-SKID-05</x:v>
+        <x:v>IAB-SKID-05</x:v>
       </x:c>
       <x:c r="E37" s="6" t="str">
         <x:v>Zone 1, Zone 2 and master E-stop stations</x:v>
@@ -1797,11 +1797,11 @@
         <x:v>SKID-05 - Safety I/O / ArmorBlock</x:v>
       </x:c>
       <x:c r="B38" s="6" t="str">
-        <x:v>IAB-20261023-SKID-05-B040</x:v>
+        <x:v>IAB-SKID-05-B040</x:v>
       </x:c>
       <x:c r="C38" s="6" t="str"/>
       <x:c r="D38" s="6" t="str">
-        <x:v>IAB-20261023-SKID-05</x:v>
+        <x:v>IAB-SKID-05</x:v>
       </x:c>
       <x:c r="E38" s="6" t="str">
         <x:v>M12 safety/standard I/O blocks at lower left</x:v>
@@ -1836,11 +1836,11 @@
         <x:v>SKID-05 - Status indicators</x:v>
       </x:c>
       <x:c r="B39" s="6" t="str">
-        <x:v>IAB-20261023-SKID-05-B050</x:v>
+        <x:v>IAB-SKID-05-B050</x:v>
       </x:c>
       <x:c r="C39" s="6" t="str"/>
       <x:c r="D39" s="6" t="str">
-        <x:v>IAB-20261023-SKID-05</x:v>
+        <x:v>IAB-SKID-05</x:v>
       </x:c>
       <x:c r="E39" s="6" t="str">
         <x:v>Zone indicator pilot lights and colored pushbuttons</x:v>
@@ -1875,11 +1875,11 @@
         <x:v>SKID-05 - Terminal block marshalling</x:v>
       </x:c>
       <x:c r="B40" s="6" t="str">
-        <x:v>IAB-20261023-SKID-05-B060</x:v>
+        <x:v>IAB-SKID-05-B060</x:v>
       </x:c>
       <x:c r="C40" s="6" t="str"/>
       <x:c r="D40" s="6" t="str">
-        <x:v>IAB-20261023-SKID-05</x:v>
+        <x:v>IAB-SKID-05</x:v>
       </x:c>
       <x:c r="E40" s="6" t="str">
         <x:v>DIN rail terminal block bank at lower right</x:v>
@@ -1914,11 +1914,11 @@
         <x:v>SKID-06 - PanelView HMI</x:v>
       </x:c>
       <x:c r="B41" s="6" t="str">
-        <x:v>IAB-20261023-SKID-06-B010</x:v>
+        <x:v>IAB-SKID-06-B010</x:v>
       </x:c>
       <x:c r="C41" s="6" t="str"/>
       <x:c r="D41" s="6" t="str">
-        <x:v>IAB-20261023-SKID-06</x:v>
+        <x:v>IAB-SKID-06</x:v>
       </x:c>
       <x:c r="E41" s="6" t="str">
         <x:v>Allen-Bradley HMI showing machine overview</x:v>
@@ -1953,11 +1953,11 @@
         <x:v>SKID-06 - Compact machine controller</x:v>
       </x:c>
       <x:c r="B42" s="6" t="str">
-        <x:v>IAB-20261023-SKID-06-B020</x:v>
+        <x:v>IAB-SKID-06-B020</x:v>
       </x:c>
       <x:c r="C42" s="6" t="str"/>
       <x:c r="D42" s="6" t="str">
-        <x:v>IAB-20261023-SKID-06</x:v>
+        <x:v>IAB-SKID-06</x:v>
       </x:c>
       <x:c r="E42" s="6" t="str">
         <x:v>PLC/controller assembly at upper center with I/O modules</x:v>
@@ -1992,11 +1992,11 @@
         <x:v>SKID-06 - Managed switch</x:v>
       </x:c>
       <x:c r="B43" s="6" t="str">
-        <x:v>IAB-20261023-SKID-06-B030</x:v>
+        <x:v>IAB-SKID-06-B030</x:v>
       </x:c>
       <x:c r="C43" s="6" t="str"/>
       <x:c r="D43" s="6" t="str">
-        <x:v>IAB-20261023-SKID-06</x:v>
+        <x:v>IAB-SKID-06</x:v>
       </x:c>
       <x:c r="E43" s="6" t="str">
         <x:v>Allen-Bradley Stratix switch visible mid-left</x:v>
@@ -2031,11 +2031,11 @@
         <x:v>SKID-06 - Linear actuator / motor load</x:v>
       </x:c>
       <x:c r="B44" s="6" t="str">
-        <x:v>IAB-20261023-SKID-06-B040</x:v>
+        <x:v>IAB-SKID-06-B040</x:v>
       </x:c>
       <x:c r="C44" s="6" t="str"/>
       <x:c r="D44" s="6" t="str">
-        <x:v>IAB-20261023-SKID-06</x:v>
+        <x:v>IAB-SKID-06</x:v>
       </x:c>
       <x:c r="E44" s="6" t="str">
         <x:v>Vertical actuator/servo or linear motion assembly on left</x:v>
@@ -2070,11 +2070,11 @@
         <x:v>SKID-06 - VFD / servo drive</x:v>
       </x:c>
       <x:c r="B45" s="6" t="str">
-        <x:v>IAB-20261023-SKID-06-B050</x:v>
+        <x:v>IAB-SKID-06-B050</x:v>
       </x:c>
       <x:c r="C45" s="6" t="str"/>
       <x:c r="D45" s="6" t="str">
-        <x:v>IAB-20261023-SKID-06</x:v>
+        <x:v>IAB-SKID-06</x:v>
       </x:c>
       <x:c r="E45" s="6" t="str">
         <x:v>Drive technology at upper right with Ethernet and power cabling</x:v>
@@ -2109,11 +2109,11 @@
         <x:v>SKID-06 - Power supply and circuit protection</x:v>
       </x:c>
       <x:c r="B46" s="6" t="str">
-        <x:v>IAB-20261023-SKID-06-B060</x:v>
+        <x:v>IAB-SKID-06-B060</x:v>
       </x:c>
       <x:c r="C46" s="6" t="str"/>
       <x:c r="D46" s="6" t="str">
-        <x:v>IAB-20261023-SKID-06</x:v>
+        <x:v>IAB-SKID-06</x:v>
       </x:c>
       <x:c r="E46" s="6" t="str">
         <x:v>DIN rail DC power supply, breakers, contactors and branch protection</x:v>
@@ -2148,11 +2148,11 @@
         <x:v>SKID-06 - Distributed I/O and terminals</x:v>
       </x:c>
       <x:c r="B47" s="6" t="str">
-        <x:v>IAB-20261023-SKID-06-B070</x:v>
+        <x:v>IAB-SKID-06-B070</x:v>
       </x:c>
       <x:c r="C47" s="6" t="str"/>
       <x:c r="D47" s="6" t="str">
-        <x:v>IAB-20261023-SKID-06</x:v>
+        <x:v>IAB-SKID-06</x:v>
       </x:c>
       <x:c r="E47" s="6" t="str">
         <x:v>Terminal block and field wiring assemblies on right</x:v>

</xml_diff>